<commit_message>
excel report final version
</commit_message>
<xml_diff>
--- a/.claude/skills/per-option-value/template/ESO template.xlsx
+++ b/.claude/skills/per-option-value/template/ESO template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tommy\Documents\Github\simple-agent\.claude\skills\per-option-value\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE2F106-D616-4469-A622-33313C37A62A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5252028D-2EE2-4140-86AC-C14F47DD9A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="1410" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-420" yWindow="1665" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="77">
   <si>
     <t>Client Name</t>
     <phoneticPr fontId="0" type="noConversion"/>
@@ -35,207 +35,256 @@
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
   <si>
-    <t>Crazy Sports Group Limited</t>
-    <phoneticPr fontId="0" type="noConversion"/>
+    <t>Valuation Date</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>A) SUMMARY</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Exhibit A-1: Valuation Summary</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remarks</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Being the Grant date of the Subject</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Valuation Purpose</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Accounting reference</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Value Basis</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fair Value</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Currency Unit</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>HKD</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>Director</t>
+  </si>
+  <si>
+    <t>Total Option Value</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Per Option Value</t>
+  </si>
+  <si>
+    <t>:</t>
+  </si>
+  <si>
+    <t>Exhibit A-2 Terms and Conditions of the Subject</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grant Date of the Subject</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Maturity Date</t>
+  </si>
+  <si>
+    <t>Exhibit A-3 Key Parameters</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Amount</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>S</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>K</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>T</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Year</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Calculated</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>V</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>%</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>With reference to the historical volatility of the Issuer (2-year daily)</t>
+  </si>
+  <si>
+    <t>R</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>With reference to HKD Sovereign Curve (2-year yield)</t>
+  </si>
+  <si>
+    <t>D</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>With reference to the historical dividend yield of the Issuer</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Exercise Multiple for Employees</t>
+  </si>
+  <si>
+    <t>With reference to exercise behavior of the relevant employees</t>
+  </si>
+  <si>
+    <t>Assumed</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>Estimated based on historical staff turnover</t>
+  </si>
+  <si>
+    <t>Total No. of Share Options Entitled to Employees</t>
+  </si>
+  <si>
+    <t>Valuation Date</t>
+  </si>
+  <si>
+    <t>replace with "Valuation Date"</t>
+  </si>
+  <si>
+    <t>replace with Employee "PerOptionValue"</t>
+  </si>
+  <si>
+    <t>replace with Director "PerOptionValue"</t>
+  </si>
+  <si>
+    <t>replace with "Grant Date of the Subject"</t>
+  </si>
+  <si>
+    <t>replace with "Total No. of Share Options Entitled to Employees"</t>
+  </si>
+  <si>
+    <t>replace with "Maturity Date"</t>
+  </si>
+  <si>
+    <t>replace with "Exercise Price"</t>
+  </si>
+  <si>
+    <t>replace with "Vesting Date"</t>
+  </si>
+  <si>
+    <t>replace with "Spot Price"</t>
+  </si>
+  <si>
+    <t>replace with "Strike Price"</t>
+  </si>
+  <si>
+    <t>replace with "Total No. of Share Options Entitled to Directors"</t>
+  </si>
+  <si>
+    <t>Exercise Price</t>
+  </si>
+  <si>
+    <t>Vesting Date</t>
+  </si>
+  <si>
+    <t>Spot Price</t>
+  </si>
+  <si>
+    <t>Strike Price</t>
+  </si>
+  <si>
+    <t>Time to Maturity</t>
+  </si>
+  <si>
+    <t>replace with "Time to Maturity"</t>
+  </si>
+  <si>
+    <t>Volatility</t>
+  </si>
+  <si>
+    <t>replace with "Volatility"</t>
+  </si>
+  <si>
+    <t>Risk-free Rate</t>
+  </si>
+  <si>
+    <t>replace with "Risk-free Rate"</t>
+  </si>
+  <si>
+    <t>Dividend Yield</t>
+  </si>
+  <si>
+    <t>replace with "Dividend Yield"</t>
+  </si>
+  <si>
+    <t>replace with "Exercise Multiple for Employees"</t>
+  </si>
+  <si>
+    <t>Pre-vesting Exit Rate</t>
+  </si>
+  <si>
+    <t>replace with "Pre-vesting Exit Rate"</t>
+  </si>
+  <si>
+    <t>Post-vesting Exit Rate</t>
+  </si>
+  <si>
+    <t>replace with "Post-vesting Exit Rate"</t>
+  </si>
+  <si>
+    <t>Time to Vest</t>
+  </si>
+  <si>
+    <t>replace with "Time to Vest"</t>
+  </si>
+  <si>
+    <t>replace with "Exercise Multiple for Director"</t>
+  </si>
+  <si>
+    <t>replace with "Client Name"</t>
   </si>
   <si>
     <t>Valuation Subject</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>30,000,000 Share Options Issued by the Client on 12 Dec 2023</t>
-  </si>
-  <si>
-    <t>Valuation Date</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>A) SUMMARY</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Exhibit A-1: Valuation Summary</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Remarks</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Being the Grant date of the Subject</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Employee</t>
-  </si>
-  <si>
-    <t>Valuation Purpose</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Accounting reference</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Value Basis</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Fair Value</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Currency Unit</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>HKD</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Results</t>
-  </si>
-  <si>
-    <t>Director</t>
-  </si>
-  <si>
-    <t>Total Option Value</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Per Option Value</t>
-  </si>
-  <si>
-    <t>:</t>
-  </si>
-  <si>
-    <t>Exhibit A-2 Terms and Conditions of the Subject</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Grant Date of the Subject</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Total No. of Share Options Entitled to Employees</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Maturity Date</t>
-  </si>
-  <si>
-    <t>Exercise Price</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vesting Date</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Exhibit A-3 Key Parameters</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Amount</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
-    <t>S</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Spot Price</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>K</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Strike Price</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>T</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Time to Maturity</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Year</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Calculated</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>V</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Volatility</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>%</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>With reference to the historical volatility of the Issuer (2-year daily)</t>
-  </si>
-  <si>
-    <t>R</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Risk-free Rate</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>With reference to HKD Sovereign Curve (2-year yield)</t>
-  </si>
-  <si>
-    <t>D</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dividend Yield</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>With reference to the historical dividend yield of the Issuer</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Exercise Multiple for Employees</t>
-  </si>
-  <si>
-    <t>With reference to exercise behavior of the relevant employees</t>
-  </si>
-  <si>
-    <t>Pre-vesting Exit Rate</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Assumed</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Post-vesting Exit Rate</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Estimated based on historical staff turnover</t>
-  </si>
-  <si>
-    <t>Time to Vest</t>
-    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>replace with "Valuation Subject"</t>
   </si>
 </sst>
 </file>
@@ -414,7 +463,7 @@
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -588,9 +637,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="40" fontId="7" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="3" applyFill="1">
@@ -920,7 +966,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="F1" s="3"/>
       <c r="G1" s="1"/>
@@ -930,7 +976,7 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -938,7 +984,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="1"/>
@@ -948,14 +994,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="5"/>
+      <c r="E3" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="F3" s="3"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -965,7 +1013,7 @@
     <row r="4" spans="1:10">
       <c r="A4" s="6"/>
       <c r="B4" s="6" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="7"/>
@@ -991,13 +1039,13 @@
     <row r="6" spans="1:10">
       <c r="A6" s="12"/>
       <c r="B6" s="6" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="7"/>
       <c r="E6" s="14"/>
       <c r="F6" s="15" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
@@ -1007,15 +1055,17 @@
     <row r="7" spans="1:10">
       <c r="A7" s="12"/>
       <c r="B7" s="17" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C7" s="18"/>
       <c r="D7" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="20"/>
+      <c r="E7" s="20" t="s">
+        <v>43</v>
+      </c>
       <c r="F7" s="21" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G7" s="22"/>
       <c r="H7" s="22"/>
@@ -1025,14 +1075,14 @@
     <row r="8" spans="1:10">
       <c r="A8" s="12"/>
       <c r="B8" s="22" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C8" s="18"/>
       <c r="D8" s="19" t="s">
         <v>1</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="22"/>
@@ -1043,14 +1093,14 @@
     <row r="9" spans="1:10">
       <c r="A9" s="12"/>
       <c r="B9" s="22" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="19" t="s">
         <v>1</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F9" s="21"/>
       <c r="G9" s="22"/>
@@ -1061,14 +1111,14 @@
     <row r="10" spans="1:10">
       <c r="A10" s="12"/>
       <c r="B10" s="22" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C10" s="18"/>
       <c r="D10" s="19" t="s">
         <v>1</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F10" s="24"/>
       <c r="G10" s="25"/>
@@ -1091,16 +1141,16 @@
     <row r="12" spans="1:10">
       <c r="A12" s="30"/>
       <c r="B12" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
@@ -1109,17 +1159,23 @@
     <row r="13" spans="1:10">
       <c r="A13" s="31"/>
       <c r="B13" s="32" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D13" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="35"/>
+      <c r="E13" s="35" t="e">
+        <f>E14*E18</f>
+        <v>#VALUE!</v>
+      </c>
       <c r="F13" s="36"/>
-      <c r="G13" s="35"/>
+      <c r="G13" s="35" t="e">
+        <f>G14*G18</f>
+        <v>#VALUE!</v>
+      </c>
       <c r="H13" s="36"/>
       <c r="I13" s="37"/>
       <c r="J13" s="38"/>
@@ -1127,17 +1183,21 @@
     <row r="14" spans="1:10" ht="15.75" thickBot="1">
       <c r="A14" s="39"/>
       <c r="B14" s="40" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="E14" s="43"/>
+        <v>18</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>44</v>
+      </c>
       <c r="F14" s="44"/>
-      <c r="G14" s="43"/>
+      <c r="G14" s="43" t="s">
+        <v>45</v>
+      </c>
       <c r="H14" s="44"/>
       <c r="I14" s="45"/>
       <c r="J14" s="46"/>
@@ -1157,35 +1217,39 @@
     <row r="16" spans="1:10">
       <c r="A16" s="12"/>
       <c r="B16" s="6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="7"/>
       <c r="E16" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F16" s="49"/>
       <c r="G16" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H16" s="16"/>
       <c r="I16" s="15" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J16" s="16"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="12"/>
       <c r="B17" s="17" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C17" s="18"/>
       <c r="D17" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E17" s="50"/>
+      <c r="E17" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="F17" s="22"/>
-      <c r="G17" s="50"/>
+      <c r="G17" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="H17" s="22"/>
       <c r="I17" s="21"/>
       <c r="J17" s="22"/>
@@ -1193,15 +1257,19 @@
     <row r="18" spans="1:10">
       <c r="A18" s="12"/>
       <c r="B18" s="22" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E18" s="51"/>
+      <c r="E18" s="51" t="s">
+        <v>47</v>
+      </c>
       <c r="F18" s="21"/>
-      <c r="G18" s="51"/>
+      <c r="G18" s="51" t="s">
+        <v>53</v>
+      </c>
       <c r="H18" s="22"/>
       <c r="I18" s="52"/>
       <c r="J18" s="22"/>
@@ -1209,15 +1277,19 @@
     <row r="19" spans="1:10">
       <c r="A19" s="12"/>
       <c r="B19" s="17" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E19" s="50"/>
+      <c r="E19" s="50" t="s">
+        <v>48</v>
+      </c>
       <c r="F19" s="21"/>
-      <c r="G19" s="50"/>
+      <c r="G19" s="50" t="s">
+        <v>48</v>
+      </c>
       <c r="H19" s="22"/>
       <c r="I19" s="22"/>
       <c r="J19" s="22"/>
@@ -1225,17 +1297,21 @@
     <row r="20" spans="1:10">
       <c r="A20" s="12"/>
       <c r="B20" s="17" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D20" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E20" s="53"/>
+      <c r="E20" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F20" s="24"/>
-      <c r="G20" s="53"/>
+      <c r="G20" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="H20" s="22"/>
       <c r="I20" s="22"/>
       <c r="J20" s="22"/>
@@ -1243,32 +1319,36 @@
     <row r="21" spans="1:10">
       <c r="A21" s="12"/>
       <c r="B21" s="17" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E21" s="20"/>
+      <c r="E21" s="20" t="s">
+        <v>50</v>
+      </c>
       <c r="F21" s="24"/>
-      <c r="G21" s="20"/>
+      <c r="G21" s="20" t="s">
+        <v>50</v>
+      </c>
       <c r="H21" s="22"/>
       <c r="I21" s="22"/>
       <c r="J21" s="22"/>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="12"/>
-      <c r="B22" s="9">
+      <c r="B22" s="9" t="e">
         <f>E24*E30</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C22" s="26"/>
       <c r="D22" s="10"/>
       <c r="E22" s="9" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
@@ -1278,18 +1358,18 @@
     <row r="23" spans="1:10">
       <c r="A23" s="12"/>
       <c r="B23" s="6" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="7"/>
       <c r="E23" s="54" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F23" s="54" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H23" s="16"/>
       <c r="I23" s="49"/>
@@ -1297,19 +1377,23 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="12" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B24" s="55" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D24" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
+      <c r="E24" s="56" t="s">
+        <v>51</v>
+      </c>
+      <c r="F24" s="56" t="s">
+        <v>51</v>
+      </c>
       <c r="G24" s="21"/>
       <c r="H24" s="57"/>
       <c r="I24" s="22"/>
@@ -1317,17 +1401,21 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="12" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="C25" s="18"/>
       <c r="D25" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
+      <c r="E25" s="56" t="s">
+        <v>52</v>
+      </c>
+      <c r="F25" s="56" t="s">
+        <v>52</v>
+      </c>
       <c r="G25" s="21"/>
       <c r="H25" s="57"/>
       <c r="I25" s="22"/>
@@ -1335,21 +1423,25 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="12" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B26" s="55" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D26" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E26" s="58"/>
-      <c r="F26" s="59"/>
+      <c r="E26" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="F26" s="58" t="s">
+        <v>59</v>
+      </c>
       <c r="G26" s="24" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="H26" s="25"/>
       <c r="I26" s="22"/>
@@ -1357,65 +1449,77 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="60" t="s">
-        <v>40</v>
+        <v>30</v>
+      </c>
+      <c r="B27" s="59" t="s">
+        <v>60</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D27" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E27" s="61"/>
-      <c r="F27" s="62"/>
+      <c r="E27" s="60" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" s="60" t="s">
+        <v>61</v>
+      </c>
       <c r="G27" s="24" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="H27" s="25"/>
       <c r="I27" s="22"/>
-      <c r="J27" s="63"/>
+      <c r="J27" s="62"/>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="B28" s="60" t="s">
-        <v>44</v>
+        <v>33</v>
+      </c>
+      <c r="B28" s="59" t="s">
+        <v>62</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D28" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E28" s="61"/>
-      <c r="F28" s="62"/>
+      <c r="E28" s="60" t="s">
+        <v>63</v>
+      </c>
+      <c r="F28" s="60" t="s">
+        <v>63</v>
+      </c>
       <c r="G28" s="24" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="H28" s="25"/>
       <c r="I28" s="22"/>
-      <c r="J28" s="63"/>
+      <c r="J28" s="62"/>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B29" s="60" t="s">
-        <v>47</v>
+        <v>35</v>
+      </c>
+      <c r="B29" s="59" t="s">
+        <v>64</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D29" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E29" s="62"/>
-      <c r="F29" s="62"/>
+      <c r="E29" s="61" t="s">
+        <v>65</v>
+      </c>
+      <c r="F29" s="61" t="s">
+        <v>65</v>
+      </c>
       <c r="G29" s="24" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="H29" s="25"/>
       <c r="I29" s="22"/>
@@ -1423,77 +1527,93 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="12"/>
-      <c r="B30" s="60" t="s">
-        <v>49</v>
+      <c r="B30" s="59" t="s">
+        <v>37</v>
       </c>
       <c r="C30" s="18"/>
       <c r="D30" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E30" s="64"/>
-      <c r="F30" s="59"/>
+      <c r="E30" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="F30" s="63" t="s">
+        <v>73</v>
+      </c>
       <c r="G30" s="24" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="H30" s="25"/>
       <c r="I30" s="22"/>
-      <c r="J30" s="65"/>
+      <c r="J30" s="64"/>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="12"/>
       <c r="B31" s="22" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D31" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E31" s="64"/>
-      <c r="F31" s="64"/>
+      <c r="E31" s="63" t="s">
+        <v>68</v>
+      </c>
+      <c r="F31" s="63" t="s">
+        <v>68</v>
+      </c>
       <c r="G31" s="24" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="H31" s="25"/>
       <c r="I31" s="22"/>
-      <c r="J31" s="63"/>
+      <c r="J31" s="62"/>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="12"/>
-      <c r="B32" s="60" t="s">
-        <v>53</v>
+      <c r="B32" s="59" t="s">
+        <v>69</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D32" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E32" s="61"/>
-      <c r="F32" s="62"/>
+      <c r="E32" s="60" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32" s="61" t="s">
+        <v>70</v>
+      </c>
       <c r="G32" s="24" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="H32" s="25"/>
       <c r="I32" s="22"/>
-      <c r="J32" s="63"/>
+      <c r="J32" s="62"/>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="12"/>
       <c r="B33" s="55" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D33" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E33" s="64"/>
-      <c r="F33" s="64"/>
+      <c r="E33" s="63" t="s">
+        <v>72</v>
+      </c>
+      <c r="F33" s="63" t="s">
+        <v>72</v>
+      </c>
       <c r="G33" s="24" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="H33" s="25"/>
       <c r="I33" s="22"/>

</xml_diff>

<commit_message>
change template to normal bg color
</commit_message>
<xml_diff>
--- a/.claude/skills/per-option-value/template/ESO template.xlsx
+++ b/.claude/skills/per-option-value/template/ESO template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tommy\Documents\Github\simple-agent\.claude\skills\per-option-value\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B816608-B53B-414A-AA9A-5EB39FB28AF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27031C9F-90DC-4D12-B5D5-ED9089B996B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="360" windowWidth="13920" windowHeight="14925" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -388,7 +388,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -409,12 +409,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -422,18 +416,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -468,7 +450,7 @@
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -518,31 +500,28 @@
     <xf numFmtId="14" fontId="4" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="2" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="3" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="2" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="38" fontId="2" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1">
+    <xf numFmtId="38" fontId="2" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
@@ -563,49 +542,49 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="6" borderId="0" xfId="4" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="0" xfId="4" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="6" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="37" fontId="3" fillId="6" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="37" fontId="3" fillId="5" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="6" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="6" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="6" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="3" fillId="5" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="6" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="6" fillId="5" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="7" fillId="5" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="6" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="7" fillId="5" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="3" applyFont="1">
@@ -617,50 +596,47 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="3" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="38" fontId="7" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="7" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="2" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="3" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="7" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="7" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="5" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="40" fontId="7" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="2" fillId="4" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="40" fontId="7" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="3" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="7" fillId="5" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="7" fillId="4" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="2" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1059,92 +1035,92 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="12"/>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" s="20" t="s">
+      <c r="C7" s="17"/>
+      <c r="D7" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="F7" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="12"/>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" s="20" t="s">
+      <c r="C8" s="17"/>
+      <c r="D8" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="21"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="12"/>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" s="20" t="s">
+      <c r="C9" s="17"/>
+      <c r="D9" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="21"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="12"/>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" s="23" t="s">
+      <c r="C10" s="17"/>
+      <c r="D10" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="12"/>
       <c r="B11" s="9"/>
-      <c r="C11" s="26"/>
+      <c r="C11" s="25"/>
       <c r="D11" s="10"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="29"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="28"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="30"/>
+      <c r="A12" s="29"/>
       <c r="B12" s="6" t="s">
         <v>13</v>
       </c>
@@ -1162,56 +1138,56 @@
       <c r="J12" s="6"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31"/>
-      <c r="B13" s="32" t="s">
+      <c r="A13" s="30"/>
+      <c r="B13" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" s="35" t="e">
+      <c r="D13" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="34" t="e">
         <f>E14*E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F13" s="36"/>
-      <c r="G13" s="35" t="e">
+      <c r="F13" s="35"/>
+      <c r="G13" s="34" t="e">
         <f>G14*G18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H13" s="36"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="38"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="37"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" thickBot="1">
-      <c r="A14" s="39"/>
-      <c r="B14" s="40" t="s">
+      <c r="A14" s="38"/>
+      <c r="B14" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="C14" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="42" t="s">
+      <c r="D14" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="43" t="s">
+      <c r="E14" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="44"/>
-      <c r="G14" s="43" t="s">
+      <c r="F14" s="43"/>
+      <c r="G14" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="H14" s="44"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="46"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="45"/>
     </row>
     <row r="15" spans="1:10" ht="15.75" thickTop="1">
       <c r="A15" s="12"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="48"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="47"/>
       <c r="E15" s="9"/>
       <c r="F15" s="11"/>
       <c r="G15" s="9"/>
@@ -1229,7 +1205,7 @@
       <c r="E16" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="49"/>
+      <c r="F16" s="48"/>
       <c r="G16" s="6" t="s">
         <v>14</v>
       </c>
@@ -1241,105 +1217,105 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="12"/>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E17" s="50" t="s">
+      <c r="C17" s="17"/>
+      <c r="D17" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="22"/>
-      <c r="G17" s="50" t="s">
+      <c r="F17" s="21"/>
+      <c r="G17" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="H17" s="22"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="22"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="21"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="12"/>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E18" s="51" t="s">
+      <c r="C18" s="17"/>
+      <c r="D18" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E18" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="F18" s="21"/>
-      <c r="G18" s="51" t="s">
+      <c r="F18" s="20"/>
+      <c r="G18" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="H18" s="22"/>
-      <c r="I18" s="52"/>
-      <c r="J18" s="22"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="21"/>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="12"/>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E19" s="50" t="s">
+      <c r="C19" s="17"/>
+      <c r="D19" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E19" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="21"/>
-      <c r="G19" s="50" t="s">
+      <c r="F19" s="20"/>
+      <c r="G19" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="12"/>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="62" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E20" s="53" t="s">
+      <c r="D20" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E20" s="52" t="s">
         <v>61</v>
       </c>
-      <c r="F20" s="24"/>
-      <c r="G20" s="53" t="s">
+      <c r="F20" s="23"/>
+      <c r="G20" s="52" t="s">
         <v>61</v>
       </c>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="12"/>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="62" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E21" s="20" t="s">
+      <c r="C21" s="17"/>
+      <c r="D21" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="24"/>
-      <c r="G21" s="20" t="s">
+      <c r="F21" s="23"/>
+      <c r="G21" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="21"/>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="12"/>
@@ -1347,7 +1323,7 @@
         <f>E24*E30</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C22" s="26"/>
+      <c r="C22" s="25"/>
       <c r="D22" s="10"/>
       <c r="E22" s="9" t="s">
         <v>7</v>
@@ -1357,8 +1333,8 @@
       </c>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="29"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="28"/>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="12"/>
@@ -1367,262 +1343,262 @@
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="7"/>
-      <c r="E23" s="54" t="s">
+      <c r="E23" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="F23" s="54" t="s">
+      <c r="F23" s="53" t="s">
         <v>23</v>
       </c>
       <c r="G23" s="15" t="s">
         <v>5</v>
       </c>
       <c r="H23" s="16"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="55" t="s">
+      <c r="B24" s="62" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E24" s="56" t="s">
+      <c r="D24" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E24" s="54" t="s">
         <v>65</v>
       </c>
-      <c r="F24" s="56" t="s">
+      <c r="F24" s="54" t="s">
         <v>65</v>
       </c>
-      <c r="G24" s="21"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="55"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E25" s="56" t="s">
+      <c r="C25" s="17"/>
+      <c r="D25" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E25" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="F25" s="56" t="s">
+      <c r="F25" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="G25" s="21"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="55" t="s">
+      <c r="B26" s="62" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E26" s="58" t="s">
+      <c r="D26" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E26" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="F26" s="58" t="s">
+      <c r="F26" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="G26" s="24" t="s">
+      <c r="G26" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="H26" s="25"/>
-      <c r="I26" s="22"/>
-      <c r="J26" s="22"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="59" t="s">
+      <c r="B27" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D27" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E27" s="60" t="s">
+      <c r="D27" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E27" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="F27" s="60" t="s">
+      <c r="F27" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="G27" s="24" t="s">
+      <c r="G27" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H27" s="25"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="62"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="59"/>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="59" t="s">
+      <c r="B28" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D28" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E28" s="60" t="s">
+      <c r="D28" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E28" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="F28" s="60" t="s">
+      <c r="F28" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="G28" s="24" t="s">
+      <c r="G28" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="25"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="62"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="59"/>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="59" t="s">
+      <c r="B29" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E29" s="61" t="s">
+      <c r="D29" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E29" s="58" t="s">
         <v>70</v>
       </c>
-      <c r="F29" s="61" t="s">
+      <c r="F29" s="58" t="s">
         <v>70</v>
       </c>
-      <c r="G29" s="24" t="s">
+      <c r="G29" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="25"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="21"/>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="12"/>
-      <c r="B30" s="59" t="s">
+      <c r="B30" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E30" s="63" t="s">
+      <c r="C30" s="17"/>
+      <c r="D30" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E30" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="F30" s="63" t="s">
+      <c r="F30" s="60" t="s">
         <v>72</v>
       </c>
-      <c r="G30" s="24" t="s">
+      <c r="G30" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="H30" s="25"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="64"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="61"/>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="12"/>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E31" s="63" t="s">
+      <c r="D31" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E31" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="F31" s="63" t="s">
+      <c r="F31" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="G31" s="24" t="s">
+      <c r="G31" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="H31" s="25"/>
-      <c r="I31" s="22"/>
-      <c r="J31" s="62"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="59"/>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="12"/>
-      <c r="B32" s="59" t="s">
+      <c r="B32" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D32" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E32" s="60" t="s">
+      <c r="D32" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E32" s="57" t="s">
         <v>78</v>
       </c>
-      <c r="F32" s="61" t="s">
+      <c r="F32" s="58" t="s">
         <v>77</v>
       </c>
-      <c r="G32" s="24" t="s">
+      <c r="G32" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="H32" s="25"/>
-      <c r="I32" s="22"/>
-      <c r="J32" s="62"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="59"/>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="12"/>
-      <c r="B33" s="55" t="s">
+      <c r="B33" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D33" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E33" s="63" t="s">
+      <c r="D33" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E33" s="60" t="s">
         <v>74</v>
       </c>
-      <c r="F33" s="63" t="s">
+      <c r="F33" s="60" t="s">
         <v>74</v>
       </c>
-      <c r="G33" s="24" t="s">
+      <c r="G33" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="H33" s="25"/>
-      <c r="I33" s="22"/>
-      <c r="J33" s="22"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add excel template, calc script. lack docx modificatioin
</commit_message>
<xml_diff>
--- a/.claude/skills/per-option-value/template/ESO template.xlsx
+++ b/.claude/skills/per-option-value/template/ESO template.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tommy\Documents\Github\simple-agent\.claude\skills\per-option-value\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27031C9F-90DC-4D12-B5D5-ED9089B996B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE3964B-9CAC-4F2C-A5FC-182414141713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4815" yWindow="6450" windowWidth="13920" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -450,7 +450,7 @@
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -634,9 +634,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyFill="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1025,17 +1022,17 @@
       <c r="C6" s="13"/>
       <c r="D6" s="7"/>
       <c r="E6" s="14"/>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="15"/>
+      <c r="G6" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="16"/>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
       <c r="J6" s="16"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="12"/>
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="17"/>
@@ -1045,10 +1042,10 @@
       <c r="E7" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="20"/>
+      <c r="G7" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="21"/>
       <c r="H7" s="21"/>
       <c r="I7" s="21"/>
       <c r="J7" s="21"/>
@@ -1129,10 +1126,10 @@
       <c r="E12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>14</v>
       </c>
+      <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
@@ -1152,11 +1149,11 @@
         <f>E14*E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F13" s="35"/>
-      <c r="G13" s="34" t="e">
-        <f>G14*G18</f>
+      <c r="F13" s="34" t="e">
+        <f>F14*F18</f>
         <v>#VALUE!</v>
       </c>
+      <c r="G13" s="34"/>
       <c r="H13" s="35"/>
       <c r="I13" s="36"/>
       <c r="J13" s="37"/>
@@ -1175,10 +1172,10 @@
       <c r="E14" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="43"/>
-      <c r="G14" s="42" t="s">
+      <c r="F14" s="42" t="s">
         <v>58</v>
       </c>
+      <c r="G14" s="42"/>
       <c r="H14" s="43"/>
       <c r="I14" s="44"/>
       <c r="J14" s="45"/>
@@ -1189,7 +1186,7 @@
       <c r="C15" s="46"/>
       <c r="D15" s="47"/>
       <c r="E15" s="9"/>
-      <c r="F15" s="11"/>
+      <c r="F15" s="9"/>
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
@@ -1205,19 +1202,19 @@
       <c r="E16" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="48"/>
-      <c r="G16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>14</v>
       </c>
+      <c r="G16" s="15" t="s">
+        <v>5</v>
+      </c>
       <c r="H16" s="16"/>
-      <c r="I16" s="15" t="s">
-        <v>5</v>
-      </c>
+      <c r="I16" s="15"/>
       <c r="J16" s="16"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="12"/>
-      <c r="B17" s="62" t="s">
+      <c r="B17" s="9" t="s">
         <v>19</v>
       </c>
       <c r="C17" s="17"/>
@@ -1227,17 +1224,17 @@
       <c r="E17" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="21"/>
-      <c r="G17" s="49" t="s">
+      <c r="F17" s="49" t="s">
         <v>59</v>
       </c>
+      <c r="G17" s="49"/>
       <c r="H17" s="21"/>
       <c r="I17" s="20"/>
       <c r="J17" s="21"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="12"/>
-      <c r="B18" s="62" t="s">
+      <c r="B18" s="9" t="s">
         <v>40</v>
       </c>
       <c r="C18" s="17"/>
@@ -1247,17 +1244,17 @@
       <c r="E18" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="F18" s="20"/>
-      <c r="G18" s="50" t="s">
+      <c r="F18" s="50" t="s">
         <v>64</v>
       </c>
+      <c r="G18" s="50"/>
       <c r="H18" s="21"/>
       <c r="I18" s="51"/>
       <c r="J18" s="21"/>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="12"/>
-      <c r="B19" s="62" t="s">
+      <c r="B19" s="9" t="s">
         <v>20</v>
       </c>
       <c r="C19" s="17"/>
@@ -1267,17 +1264,17 @@
       <c r="E19" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="20"/>
-      <c r="G19" s="49" t="s">
+      <c r="F19" s="49" t="s">
         <v>60</v>
       </c>
+      <c r="G19" s="49"/>
       <c r="H19" s="21"/>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="12"/>
-      <c r="B20" s="62" t="s">
+      <c r="B20" s="9" t="s">
         <v>42</v>
       </c>
       <c r="C20" s="17" t="s">
@@ -1289,17 +1286,17 @@
       <c r="E20" s="52" t="s">
         <v>61</v>
       </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="52" t="s">
+      <c r="F20" s="52" t="s">
         <v>61</v>
       </c>
+      <c r="G20" s="52"/>
       <c r="H20" s="21"/>
       <c r="I20" s="21"/>
       <c r="J20" s="21"/>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="12"/>
-      <c r="B21" s="62" t="s">
+      <c r="B21" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C21" s="17"/>
@@ -1309,10 +1306,10 @@
       <c r="E21" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="23"/>
-      <c r="G21" s="19" t="s">
+      <c r="F21" s="19" t="s">
         <v>62</v>
       </c>
+      <c r="G21" s="19"/>
       <c r="H21" s="21"/>
       <c r="I21" s="21"/>
       <c r="J21" s="21"/>
@@ -1360,7 +1357,7 @@
       <c r="A24" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="62" t="s">
+      <c r="B24" s="9" t="s">
         <v>44</v>
       </c>
       <c r="C24" s="17" t="s">
@@ -1384,7 +1381,7 @@
       <c r="A25" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="62" t="s">
+      <c r="B25" s="9" t="s">
         <v>45</v>
       </c>
       <c r="C25" s="17"/>
@@ -1406,7 +1403,7 @@
       <c r="A26" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="62" t="s">
+      <c r="B26" s="9" t="s">
         <v>46</v>
       </c>
       <c r="C26" s="17" t="s">
@@ -1432,7 +1429,7 @@
       <c r="A27" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="62" t="s">
+      <c r="B27" s="9" t="s">
         <v>47</v>
       </c>
       <c r="C27" s="17" t="s">
@@ -1458,7 +1455,7 @@
       <c r="A28" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="62" t="s">
+      <c r="B28" s="9" t="s">
         <v>48</v>
       </c>
       <c r="C28" s="17" t="s">
@@ -1484,7 +1481,7 @@
       <c r="A29" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="62" t="s">
+      <c r="B29" s="9" t="s">
         <v>49</v>
       </c>
       <c r="C29" s="17" t="s">
@@ -1508,7 +1505,7 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="12"/>
-      <c r="B30" s="62" t="s">
+      <c r="B30" s="9" t="s">
         <v>36</v>
       </c>
       <c r="C30" s="17"/>
@@ -1530,7 +1527,7 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="12"/>
-      <c r="B31" s="62" t="s">
+      <c r="B31" s="9" t="s">
         <v>50</v>
       </c>
       <c r="C31" s="17" t="s">
@@ -1554,7 +1551,7 @@
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="12"/>
-      <c r="B32" s="62" t="s">
+      <c r="B32" s="9" t="s">
         <v>51</v>
       </c>
       <c r="C32" s="17" t="s">
@@ -1578,7 +1575,7 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="12"/>
-      <c r="B33" s="62" t="s">
+      <c r="B33" s="9" t="s">
         <v>52</v>
       </c>
       <c r="C33" s="17" t="s">

</xml_diff>